<commit_message>
Added solution for #1, fixed some formatting
Used alternate borders to highlight the pineapple break triplets

modified col width for bar so table takes up less space

fixed footnotes by using row index
</commit_message>
<xml_diff>
--- a/songs.xlsx
+++ b/songs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/u1152038/Documents/local/raiodesol/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/u1152038/Documents/GitHub/raiodesol/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D41E72D-45D7-3A4F-95E9-7CC8DBCDE29A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF394F46-599C-C84C-9E67-998093B69082}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17180" xr2:uid="{592AD3B0-70B5-0648-81EC-897D5B2099BE}"/>
+    <workbookView xWindow="1100" yWindow="760" windowWidth="28040" windowHeight="17180" xr2:uid="{592AD3B0-70B5-0648-81EC-897D5B2099BE}"/>
   </bookViews>
   <sheets>
     <sheet name="london school" sheetId="1" r:id="rId1"/>
@@ -1676,22 +1676,22 @@
       <c r="D20" t="s">
         <v>17</v>
       </c>
+      <c r="F20" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20" t="s">
+        <v>17</v>
+      </c>
       <c r="H20" t="s">
         <v>17</v>
       </c>
-      <c r="I20" t="s">
-        <v>17</v>
-      </c>
-      <c r="J20" t="s">
+      <c r="K20" t="s">
         <v>17</v>
       </c>
       <c r="L20" t="s">
         <v>17</v>
       </c>
       <c r="M20" t="s">
-        <v>17</v>
-      </c>
-      <c r="N20" t="s">
         <v>17</v>
       </c>
       <c r="P20" t="s">

</xml_diff>